<commit_message>
Clarify EETT is Word document, not Excel; update Plantilla 03
- btn-ptl-03 in "Plantillas para estudiantes" now shows an explanatory
  toast: EETT is delivered as a modified Word document (yellow highlights
  for additions, strikethrough for deletions), not as an Excel file
- "Descargar plantilla/datos" in the EETT tab renamed to
  "Descargar resumen auxiliar" to distinguish the professor's companion
  Excel from the primary Word deliverable
- Plantilla 03 Excel regenerated with a prominent yellow-background note
  (row 1) that the primary deliverable is the Word document, and with
  richer DETALLE examples showing the expected level of specificity:
  calidad, marca, modelo, formato, color, proveedor (e.g. lana mineral
  AislánGlass Volcán 50mm, hormigón H-25 Melco árido máx 20mm, etc.)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016thVVhhF2qFDaoBQvgNiZf
</commit_message>
<xml_diff>
--- a/webapp/plantillas/03_Especificaciones_Tecnicas.xlsx
+++ b/webapp/plantillas/03_Especificaciones_Tecnicas.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,9 +27,9 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="005A5248"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="007A4E00"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -41,13 +41,24 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="005A5248"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -83,16 +94,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,18 +473,18 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="72" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plantilla 03 · Especificaciones Técnicas Modificadas — Formulación de Proyecto de Título · Universidad Viña del Mar</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>IMPORTANTE · Las EETT se entregan en formato WORD, no en este Excel. El estudiante recibe el documento Word base del proyecto y lo modifica resaltando en AMARILLO las adiciones y TACHANDO las eliminaciones, indicando calidad, materialidad, tipo, formato, color, modelo y marca/proveedor para cada material — sin dejar nada a interpretación. Este Excel es solo un RESUMEN AUXILIAR que el profesor completa al revisar el Word.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ITEM</t>
@@ -481,12 +492,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DETALLE</t>
+          <t>DETALLE DE LA MODIFICACIÓN (calidad · marca · modelo · formato · color · proveedor)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>MARCADO</t>
+          <t>MARCADO EN WORD</t>
         </is>
       </c>
     </row>
@@ -537,7 +548,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Resistencia característica mínima f'c=25 MPa (H-25); árido máximo 20 mm; asentamiento de cono 8-10 cm.</t>
+          <t>Aislación lana mineral AislánGlass del proveedor Volcán; espesor 50 mm en formato rollo libre, tipo R100 con resistencia térmica 188 [m²·°K/W]; color natural/beige.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -554,7 +565,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Acero A63-42H fy=420 MPa; diámetro ø8 mm.</t>
+          <t>Hormigón H-25 premezclado del proveedor Melco; árido máximo 20 mm; asentamiento de cono 8–10 cm; resistencia característica f'c = 25 MPa (250 kg/cm²).</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -597,7 +608,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Porcelanato rectificado 60×60 cm, absorción ≤0,1%, clase PEI IV; marca PORCELANITE modelo URBAN GREY 6060.</t>
+          <t>Porcelanato rectificado 60×60 cm, absorción ≤0,1%, clase PEI IV; marca PORCELANITE modelo URBAN GREY 6060; color gris oscuro mate.</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -627,7 +638,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Tablero bifásico 12 circuitos 63A; marca SCHNEIDER Electric modelo Easy9; incluye diferencial 2×40A 30mA.</t>
+          <t>Tablero bifásico 12 circuitos 63 A; marca SCHNEIDER Electric modelo Easy9 EZ9E212S2P; incluye diferencial 2×40 A 30 mA; color blanco.</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -649,10 +660,10 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="72" customHeight="1">
+    <row r="15" ht="80" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>INSTRUCCIONES: ITEM debe coincidir exactamente con los códigos del Listado de Actividades (Plantilla 01). DETALLE: describe la especificación modificada — calidad, marca, modelo, formato, color, norma, etc. Solo completa las partidas cuya especificación difiere de la EETT base del proyecto. MARCADO: SI si resaltaste el cambio en el documento Word; NO si aún no lo has marcado. Deja DETALLE vacío en las partidas que no tienen modificación de especificación.</t>
+          <t>INSTRUCCIONES (resumen auxiliar): ITEM debe coincidir con los códigos del Listado de Actividades (Plantilla 01). DETALLE: anota la especificación modificada con todos los atributos: calidad, materialidad, tipo, formato, color, modelo y marca/proveedor — sin dejar nada a interpretación, tal como aparece resaltado en el documento Word. MARCADO EN WORD: SI cuando la modificación ya está resaltada en amarillo (adición) o tachada (eliminación) en el Word; NO si aún no lo has marcado. Deja DETALLE vacío en partidas sin modificación de especificación.</t>
         </is>
       </c>
     </row>

</xml_diff>